<commit_message>
feat : load world animation
</commit_message>
<xml_diff>
--- a/ModelEditor/AnimationName.xlsx
+++ b/ModelEditor/AnimationName.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="Polaris Office Sheet" lastEdited="6" lowestEdited="6" rupBuild="10.105.298.56155"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="30" windowWidth="25755" windowHeight="11595" activeTab="0"/>
+    <workbookView xWindow="360" yWindow="30" windowWidth="25755" windowHeight="11595" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="구스타브" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>FModel기반 네이밍</t>
   </si>
@@ -97,6 +97,9 @@
   </si>
   <si>
     <t>Noah_Dash_Out</t>
+  </si>
+  <si>
+    <t>루네 시작 마엘거 씀</t>
   </si>
 </sst>
 </file>
@@ -712,7 +715,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -735,12 +738,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1077,10 +1074,10 @@
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="8" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1093,10 +1090,10 @@
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="7" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1134,17 +1131,17 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="7" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1190,10 +1187,10 @@
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="7" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat : idle 데이터 정리
</commit_message>
<xml_diff>
--- a/ModelEditor/AnimationName.xlsx
+++ b/ModelEditor/AnimationName.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="Polaris Office Sheet" lastEdited="6" lowestEdited="6" rupBuild="10.105.298.56155"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="30" windowWidth="25755" windowHeight="11595" activeTab="0"/>
+    <workbookView xWindow="360" yWindow="30" windowWidth="25755" windowHeight="11595" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="구스타브" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
   <si>
     <t>FModel기반 네이밍</t>
   </si>
@@ -130,6 +130,63 @@
   </si>
   <si>
     <t>구스타브 고유 idle 모션</t>
+  </si>
+  <si>
+    <t>Idles_Lune_Break_LookAround_02</t>
+  </si>
+  <si>
+    <t>Lune_Idles_Sciel_Break_ArmsInFront_01</t>
+  </si>
+  <si>
+    <t>Lune_Idles_Sciel_Break_LookBehind</t>
+  </si>
+  <si>
+    <t>LuneBody_Anim_Lune_Idle_World</t>
+  </si>
+  <si>
+    <t>Idles_Lune_Break_HandOnHips</t>
+  </si>
+  <si>
+    <t>Idle series / 돌아보기</t>
+  </si>
+  <si>
+    <t xml:space="preserve">앞에 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">힙 </t>
+  </si>
+  <si>
+    <t>주변 돌아보기</t>
+  </si>
+  <si>
+    <t>기본 Idle</t>
+  </si>
+  <si>
+    <t>Idle series / 주변 돌아보기</t>
+  </si>
+  <si>
+    <t>뒤 체크</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Idle series </t>
+  </si>
+  <si>
+    <t>Maelle_World_Idle_V2</t>
+  </si>
+  <si>
+    <t>Idles_dust_off_Maelle</t>
+  </si>
+  <si>
+    <t>Maelle_Idles_Break_HandsOnHips</t>
+  </si>
+  <si>
+    <t>Maelle_Idles_dust_off</t>
+  </si>
+  <si>
+    <t>Maelle_Idles_look_around_02</t>
+  </si>
+  <si>
+    <t>Maelle_Idles_Sciel_Break_ArmsInFront_01</t>
   </si>
 </sst>
 </file>
@@ -1177,7 +1234,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="16.500000"/>
   <cols>
     <col min="1" max="1" style="2" width="42.38000107" customWidth="1" outlineLevel="0"/>
@@ -1215,6 +1272,49 @@
       <c r="B4" s="7" t="s">
         <v>11</v>
       </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -1226,7 +1326,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="16.500000"/>
   <cols>
     <col min="1" max="1" style="2" width="42.38000107" customWidth="1" outlineLevel="0"/>
@@ -1265,6 +1365,34 @@
         <v>11</v>
       </c>
     </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.70" right="0.70" top="0.75" bottom="0.75" header="0.30" footer="0.30"/>

</xml_diff>